<commit_message>
update uk to 2026q1
</commit_message>
<xml_diff>
--- a/data-raw/uk/epu.xlsx
+++ b/data-raw/uk/epu.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="343" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="348" uniqueCount="33">
   <si>
     <t>year</t>
   </si>
@@ -157,7 +157,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C341"/>
+  <dimension ref="A1:C346"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3897,15 +3897,70 @@
         <v>3</v>
       </c>
       <c r="C340" s="1">
-        <v>319.77885030933476</v>
+        <v>310.82265819928256</v>
       </c>
     </row>
     <row r="341">
       <c r="A341" t="s">
+        <v>29</v>
+      </c>
+      <c r="B341" s="1">
+        <v>4</v>
+      </c>
+      <c r="C341" s="1">
+        <v>309.34203033248792</v>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" t="s">
+        <v>29</v>
+      </c>
+      <c r="B342" s="1">
+        <v>5</v>
+      </c>
+      <c r="C342" s="1">
+        <v>301.63959873983106</v>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" t="s">
+        <v>29</v>
+      </c>
+      <c r="B343" s="1">
+        <v>6</v>
+      </c>
+      <c r="C343" s="1">
+        <v>207.98421936625263</v>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" t="s">
+        <v>29</v>
+      </c>
+      <c r="B344" s="1">
+        <v>7</v>
+      </c>
+      <c r="C344" s="1">
+        <v>232.13539796257373</v>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" t="s">
+        <v>29</v>
+      </c>
+      <c r="B345" s="1">
+        <v>8</v>
+      </c>
+      <c r="C345" s="1">
+        <v>250.41035828955552</v>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" t="s">
         <v>30</v>
       </c>
-      <c r="B341" s="1"/>
-      <c r="C341" s="1"/>
+      <c r="B346" s="1"/>
+      <c r="C346" s="1"/>
     </row>
   </sheetData>
 </worksheet>

</xml_diff>